<commit_message>
problems of updating effect sizes and coding interaction effects seems to be solved, but now adding an effect size instance seems to wipe the previous clean
</commit_message>
<xml_diff>
--- a/tests/test_outputs/meta_export_20260228.xlsx
+++ b/tests/test_outputs/meta_export_20260228.xlsx
@@ -351,10 +351,601 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:CN2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1"/>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>article_num</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>doi_clean</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>review_status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>reviewed_by</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>reviewed_at</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>location_osm</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>bounding_box_label</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>habitat_type</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>country_name</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>is_experimental</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>group_name</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>group_instance</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>site_name</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>test_multi</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>test_date</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>yi</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>effect_status</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>raw_n</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>raw_df</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>raw_sd_X</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>raw_sd_Y</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>raw_se_r</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>raw_t_stat</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>raw_r_reported</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>raw_study_design</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>raw_study_method</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>raw_covariance_XY</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>raw_response_unit</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>raw_predictor_unit</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_response_scale</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>raw_interaction_effect</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>raw_response_distribution</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>raw_predictor_distribution</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>raw_response_variable_name</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>raw_predictor_variable_name</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>raw_F_stat</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_p_value</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>raw_n_control</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>raw_n_treatment</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>raw_mean_control</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>raw_mean_treatment</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>raw_chi_square_stat</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>raw_var_value_control</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>raw_var_statistic_type</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>raw_control_description</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_use_small_sd_approx</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>raw_var_value_treatment</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>raw_treatment_description</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>raw_beta</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>raw_se_beta</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>raw_multiple_predictors</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>raw_beta_type</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>raw_n_predictors</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_df</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_F_stat</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_t_stat</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_p_value</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_n_control</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_n_treatment</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_mean_control</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_study_design</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_mean_treatment</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_chi_square_stat</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_var_value_control</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_var_statistic_type</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_control_description</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_use_small_sd_approx</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_var_value_treatment</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_a_treatment_description</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_df</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_F_stat</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_t_stat</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_p_value</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_n_control</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_n_treatment</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_mean_control</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_study_design</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_mean_treatment</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_chi_square_stat</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_var_value_control</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_var_statistic_type</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_control_description</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_use_small_sd_approx</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_var_value_treatment</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>raw_group_b_treatment_description</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>raw_interaction_pathway</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Huang JX; Torres MM; Eriksen S</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>2020</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10.1007/s10750-020-04321-y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>564c9186-f70d-47f2-b285-55baee74f705</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-02-28T15:25:37+00:00</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Grassland</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>study_site</t>
+        </is>
+      </c>
+      <c r="P2">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Test effect size 2</t>
+        </is>
+      </c>
+      <c r="T2">
+        <v>0.8</v>
+      </c>
+      <c r="U2">
+        <v>1.09861228866811</v>
+      </c>
+      <c r="V2">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>correlation</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Experimental (ex-situ)</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Ind. behaviour</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>